<commit_message>
Dopasowanie klubow i nazwy lig: nazwy klubow z Transfermarktu mapowane na nazwy z API (m.in. OH Leuven, Benfica, Slavia, Dynamo Kyiv, Rennes); serwer ustala nazwe nieznanej ligi od razu, nie po meczu; nowe ID Championship; KuPS Akatemia jako rezerwy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/zawodnicy.xlsx
+++ b/zawodnicy.xlsx
@@ -752,7 +752,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>[Mołdawia] FC Milsami Orgiejów</t>
+          <t>[Mołdawia] FC Milsami Orhei</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>[Czechy] FK Dukla Praga</t>
+          <t>[Czechy] Dukla Praha</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>[Francja] Stade Rennais FC</t>
+          <t>[Francja] Rennes</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>[Portugalia] Benfika Lizbona</t>
+          <t>[Portugalia] Benfica</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>[Niemcy] Rot-Weiss Essen</t>
+          <t>[Niemcy] RW Essen</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>[Czechy] SK Slavia Praga</t>
+          <t>[Czechy] Slavia Prague</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>[Ukraina] Dynamo Kijów</t>
+          <t>[Ukraina] Dynamo Kyiv</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>[Belgia] Oud-Heverlee Leuven</t>
+          <t>[Belgia] OH Leuven</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>[Cypr] Omonia Nikozja</t>
+          <t>[Cypr] Omonia Nicosia</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>[Czechy] SK Slavia Praga</t>
+          <t>[Czechy] Slavia Prague</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>[Finlandia] Kuopion Palloseura</t>
+          <t>[Finlandia] KuPS</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>[Turcja] Igdir FK</t>
+          <t>[Turcja] Iğdır FK</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>[Francja] Stade Rennais FC</t>
+          <t>[Francja] Rennes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nacje: Pakistanczycy (land_id 128); skaner: zawodnik bez linku do ligi (amatorskie, regionalne ligi) pomijany - wczesniej liczyl sie jako 1. poziom; kluby "X Reserves" i ligi kobiece z meskimi nazwami druzyn (szkocka SWPL, Kvinner, Vrouwen, Liga F...) odfiltrowane; daty dopisania zawodnikow porownywane bez polskich znakow (Michal/Michał Helik); swieze bazy wszystkich nacji; limit workflow 60 min
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/zawodnicy.xlsx
+++ b/zawodnicy.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -963,7 +963,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Michal</t>
+          <t>Michał</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1133,765 +1133,765 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dawid</t>
+          <t>Kacper</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Kownacki</t>
+          <t>Kozłowski</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>[Niemcy] SV Werder Bremen</t>
+          <t>[Turcja] Gaziantep FK</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kacper</t>
+          <t>Oskar</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Kozłowski</t>
+          <t>Kubiak</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>[Turcja] Gaziantep FK</t>
+          <t>[Czechy] Slavia Prague</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Oskar</t>
+          <t>Dawid</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Kubiak</t>
+          <t>Kurminowski</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>[Czechy] Slavia Prague</t>
+          <t>[Grecja] Kalamata FC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Dawid</t>
+          <t>Krzysztof</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Kurminowski</t>
+          <t>Kurowski</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>[Grecja] Kalamata FC</t>
+          <t>[Holandia] FC Twente Enschede</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Krzysztof</t>
+          <t>Tomasz</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Kurowski</t>
+          <t>Kędziora</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>[Holandia] FC Twente Enschede</t>
+          <t>[Ukraina] Dynamo Kyiv</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tomasz</t>
+          <t>Oskar</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Kędziora</t>
+          <t>Lachowicz</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>[Ukraina] Dynamo Kyiv</t>
+          <t>[Słowacja] FC ViOn Zlate Moravce-Vrable</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Oskar</t>
+          <t>Lukasz</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Lachowicz</t>
+          <t>Lakomy</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>[Słowacja] FC ViOn Zlate Moravce-Vrable</t>
+          <t>[Belgia] OH Leuven</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Lukasz</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Lakomy</t>
+          <t>Leszczyński</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>[Belgia] OH Leuven</t>
+          <t>[Niemcy] Borussia Mönchengladbach</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Robert</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Leszczyński</t>
+          <t>Lewandowski</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>[Niemcy] Borussia Mönchengladbach</t>
+          <t>[Stany Zjednaczone] Chicago Fire FC</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Patryk</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Lewandowski</t>
+          <t>Lipski</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>[Stany Zjednaczone] Chicago Fire FC</t>
+          <t>[Zjednaczone Emiraty Arabskie] Al-Fujairah SC</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Patryk</t>
+          <t>Robin</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Lipski</t>
+          <t>Lisewski</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>[Zjednaczone Emiraty Arabskie] Al-Fujairah SC</t>
+          <t>[Niemcy] 1.FC Nürnberg</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Kornel</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Lisewski</t>
+          <t>Lisman</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>[Niemcy] 1.FC Nürnberg</t>
+          <t>[Włochy] Venezia FC</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Kornel</t>
+          <t>Franciszek</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Lisman</t>
+          <t>Liszka</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>[Włochy] Venezia FC</t>
+          <t>[Słowacja] MSK Povazska Bystrica</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Franciszek</t>
+          <t>Maik</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Liszka</t>
+          <t>Lukowicz</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>[Słowacja] MSK Povazska Bystrica</t>
+          <t>[Zjednaczone Emiraty Arabskie] Dibba Al-Hisn SC</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Aleksander</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Lubik</t>
+          <t>Majchrzak</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>[Malta] Tarxien Rainbows</t>
+          <t>[Niemcy] VfB Stuttgart II</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Maik</t>
+          <t>Radoslaw</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Lukowicz</t>
+          <t>Majecki</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>[Zjednaczone Emiraty Arabskie] Dibba Al-Hisn SC</t>
+          <t>[Cypr] Pafos FC</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Dominik</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Majchrzak</t>
+          <t>Marczuk</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>[Niemcy] VfB Stuttgart II</t>
+          <t>[Stany Zjednaczone] Real Salt Lake City</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Radoslaw</t>
+          <t>Wiktor</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Majecki</t>
+          <t>Matyjewicz</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>[Cypr] Pafos FC</t>
+          <t>[Grecja] Athens Kallithea</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Dominik</t>
+          <t>Miłosz</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Marczuk</t>
+          <t>Matysik</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>[Stany Zjednaczone] Real Salt Lake City</t>
+          <t>[Cypr] Aris Limassol</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Wiktor</t>
+          <t>Bartosz</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Matyjewicz</t>
+          <t>Mazurek</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>[Grecja] Athens Kallithea</t>
+          <t>[Austria] Red Bull Salzburg</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Miłosz</t>
+          <t>Konrad</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Matysik</t>
+          <t>Michalak</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>[Cypr] Aris Limassol</t>
+          <t>[Turcja] Eyüpspor</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Bartosz</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Mazurek</t>
+          <t>Mikolajewski</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>[Austria] Red Bull Salzburg</t>
+          <t>[Szwajcaria] FC Luzern</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Konrad</t>
+          <t>Arkadiusz</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Michalak</t>
+          <t>Milik</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>[Turcja] Eyüpspor</t>
+          <t>[Włochy] Juventus Turyn</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Daniel</t>
+          <t>Cezary</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Mikolajewski</t>
+          <t>Miszta</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>[Szwajcaria] FC Luzern</t>
+          <t>[Portugalia] Rió Ave FC</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Arkadiusz</t>
+          <t>Jakub</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Milik</t>
+          <t>Moder</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>[Włochy] Juventus Turyn</t>
+          <t>[Holandia] Feyenoord Rotterdam</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Cezary</t>
+          <t>Pascal</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Miszta</t>
+          <t>Mozie</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>[Portugalia] Rió Ave FC</t>
+          <t>[Francja] FC Annecy</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Jakub</t>
+          <t>Bartosz</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Moder</t>
+          <t>Mrozek</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>[Holandia] Feyenoord Rotterdam</t>
+          <t>[Włochy] Udinese Calcio</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Pascal</t>
+          <t>Fabian</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Mozie</t>
+          <t>Mrozek</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>[Francja] FC Annecy</t>
+          <t>[Stany Zjednaczone] FC Cincinnati</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Bartosz</t>
+          <t>Mateusz</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Mrozek</t>
+          <t>Musiałowski</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>[Włochy] Udinese Calcio</t>
+          <t>[Cypr] Omonia Nicosia</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Fabian</t>
+          <t>Maik</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Mrozek</t>
+          <t>Nawrocki</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>[Stany Zjednaczone] FC Cincinnati</t>
+          <t>[Francja] RC Lens</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Mateusz</t>
+          <t>Wiktor</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Musiałowski</t>
+          <t>Nowak</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>[Cypr] Omonia Nicosia</t>
+          <t>[Czechy] Slavia Prague</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Maik</t>
+          <t>Jakub</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Nawrocki</t>
+          <t>Ojrzynski</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>[Francja] RC Lens</t>
+          <t>[Szwecja] Örebro SK</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Wiktor</t>
+          <t>Maxi</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Nowak</t>
+          <t>Oyedele</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>[Czechy] Slavia Prague</t>
+          <t>[Francja] RC Strasbourg Alsace</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Jakub</t>
+          <t>Piotr</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Ojrzynski</t>
+          <t>Parzyszek</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>[Szwecja] Örebro SK</t>
+          <t>[Finlandia] KuPS</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Maxi</t>
+          <t>Patryk</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Oyedele</t>
+          <t>Peda</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>[Francja] RC Strasbourg Alsace</t>
+          <t>[Włochy] Palermo FC</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Piotr</t>
+          <t>Krzysztof</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Parzyszek</t>
+          <t>Piatek</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>[Finlandia] KuPS</t>
+          <t>[Katar] Al-Duhail SC</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Patryk</t>
+          <t>Milosz</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Peda</t>
+          <t>Piekutowski</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>[Włochy] Palermo FC</t>
+          <t>[Francja] RC Strasbourg Alsace</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Krzysztof</t>
+          <t>Oskar</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Piatek</t>
+          <t>Pietuszewski</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>[Katar] Al-Duhail SC</t>
+          <t>[Portugalia] FC Porto</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Milosz</t>
+          <t>Jakub</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Piekutowski</t>
+          <t>Piotrowski</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>[Francja] RC Strasbourg Alsace</t>
+          <t>[Włochy] Udinese Calcio</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Oskar</t>
+          <t>David</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Pietuszewski</t>
+          <t>Poreba</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>[Portugalia] FC Porto</t>
+          <t>[Stany Zjednaczone] Chicago Fire FC</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Jakub</t>
+          <t>Lukasz</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Piotrowski</t>
+          <t>Poreba</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>[Włochy] Udinese Calcio</t>
+          <t>[Niemcy] SV 07 Elversberg</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Albert</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Poreba</t>
+          <t>Posiadala</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>[Stany Zjednaczone] Chicago Fire FC</t>
+          <t>[Norwegia] Molde FK</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Lukasz</t>
+          <t>Kacper</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Poreba</t>
+          <t>Potulski</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>[Niemcy] SV 07 Elversberg</t>
+          <t>[Niemcy] 1.FSV Mainz 05</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Albert</t>
+          <t>Adrian</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Posiadala</t>
+          <t>Przyborek</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>[Norwegia] Molde FK</t>
+          <t>[Włochy] Lazio Rzym</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Kacper</t>
+          <t>Tymoteusz</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Potulski</t>
+          <t>Puchacz</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>[Niemcy] 1.FSV Mainz 05</t>
+          <t>[Azerbejdżan] Sabah FK</t>
         </is>
       </c>
     </row>
@@ -1903,741 +1903,707 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Przyborek</t>
+          <t>Purzycki</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>[Włochy] Lazio Rzym</t>
+          <t>[Indonezja] PSIM Yogyakarta</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Tymoteusz</t>
+          <t>Arkadiusz</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Puchacz</t>
+          <t>Pyrka</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>[Azerbejdżan] Sabah FK</t>
+          <t>[Niemcy] FC St. Pauli</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Adrian</t>
+          <t>Przemysław</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Purzycki</t>
+          <t>Płacheta</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>[Indonezja] PSIM Yogyakarta</t>
+          <t>[Stany Zjednaczone] Austin FC</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Arkadiusz</t>
+          <t>Michal</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Pyrka</t>
+          <t>Rosiak</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>[Niemcy] FC St. Pauli</t>
+          <t>[Holandia] FC Twente Enschede</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Przemysław</t>
+          <t>Filip</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Płacheta</t>
+          <t>Rózga</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>[Stany Zjednaczone] Austin FC</t>
+          <t>[Austria] SK Sturm Graz</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Michal</t>
+          <t>Dominik</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Rosiak</t>
+          <t>Sarapata</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>[Holandia] FC Twente Enschede</t>
+          <t>[Czechy] SK Artis Brno</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Filip</t>
+          <t>Kacper</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Rózga</t>
+          <t>Sezonienko</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>[Austria] SK Sturm Graz</t>
+          <t>[Włochy] Hellas Verona</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Dominik</t>
+          <t>Michal</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Sarapata</t>
+          <t>Skoras</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>[Czechy] SK Artis Brno</t>
+          <t>[Francja] RC Lens</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Kacper</t>
+          <t>Lukasz</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Sezonienko</t>
+          <t>Skorupski</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>[Włochy] Hellas Verona</t>
+          <t>[Włochy] FC Bologna</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Michal</t>
+          <t>Konrad</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Skoras</t>
+          <t>Skuza</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>[Francja] RC Lens</t>
+          <t>[Gibraltar] Lions Gibraltar FC</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Lukasz</t>
+          <t>Oskar</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Skorupski</t>
+          <t>Skuza</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>[Włochy] FC Bologna</t>
+          <t>[Gibraltar] FC Hound Dogs</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Konrad</t>
+          <t>Bartosz</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Skuza</t>
+          <t>Slisz</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>[Gibraltar] Lions Gibraltar FC</t>
+          <t>[Dania] Bröndby IF</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Oskar</t>
+          <t>Jakub</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Skuza</t>
+          <t>Slowik</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>[Gibraltar] FC Hound Dogs</t>
+          <t>[Japonia] Mito HollyHock</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Bartosz</t>
+          <t>Maciej</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Slisz</t>
+          <t>Soboczynski</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>[Dania] Bröndby IF</t>
+          <t>[Norwegia] Rosenborg BK</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Jakub</t>
+          <t>Dariusz</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Slowik</t>
+          <t>Stalmach</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>[Japonia] Mito HollyHock</t>
+          <t>[Niemcy] SV Werder Bremen</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Maciej</t>
+          <t>Adrian</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Soboczynski</t>
+          <t>Stanilewicz</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>[Norwegia] Rosenborg BK</t>
+          <t>[Niemcy] SC Fortuna Köln</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Dariusz</t>
+          <t>Jakub</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Stalmach</t>
+          <t>Stolarczyk</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>[Niemcy] SV Werder Bremen</t>
+          <t>[Anglia] Leicester City</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Adrian</t>
+          <t>Maksymilian</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Stanilewicz</t>
+          <t>Stryjek</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>[Niemcy] SC Fortuna Köln</t>
+          <t>[Szkocja] Kilmarnock FC</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Jakub</t>
+          <t>Wojciech</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Stolarczyk</t>
+          <t>Szczęsny</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>[Anglia] Leicester City</t>
+          <t>[Hiszpania] FC Barcelona</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Maksymilian</t>
+          <t>Oskar</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Stryjek</t>
+          <t>Szulc</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>[Szkocja] Kilmarnock FC</t>
+          <t>[Belgia] FCV Dender EH</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Wojciech</t>
+          <t>Jakub</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Szczesny</t>
+          <t>Szumski</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>[Hiszpania] FC Barcelona</t>
+          <t>[Turcja] Iğdır FK</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Oskar</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Szulc</t>
+          <t>Szymański</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>[Belgia] FCV Dender EH</t>
+          <t>[Francja] Rennes</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Jakub</t>
+          <t>Bartosz</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Szumski</t>
+          <t>Szywala</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>[Turcja] Iğdır FK</t>
+          <t>[Czechy] SK Slavia Praga B</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Kacper</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Szymański</t>
+          <t>Tobiasz</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>[Francja] Rennes</t>
+          <t>[Turcja] Gaziantep FK</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Bartosz</t>
+          <t>Milosz</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Szywala</t>
+          <t>Trojak</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>[Czechy] SK Slavia Praga B</t>
+          <t>[Korea Południowa] Ulsan HD FC</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Kacper</t>
+          <t>Damian</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Tobiasz</t>
+          <t>Vu Thanh</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>[Turcja] Gaziantep FK</t>
+          <t>[Wietnam] The Cong - Viettel FC</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Milosz</t>
+          <t>Tomasz</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Trojak</t>
+          <t>Walczak</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>[Korea Południowa] Ulsan HD FC</t>
+          <t>[Słowacja] Zemplin Michalovce</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Damian</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Vu Thanh</t>
+          <t>Walukiewicz</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>[Wietnam] The Cong - Viettel FC</t>
+          <t>[Włochy] US Sassuolo</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Tomasz</t>
+          <t>Jakub</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Walczak</t>
+          <t>Wawszczyk</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>[Słowacja] Zemplin Michalovce</t>
+          <t>[Litwa] FC Džiugas Telšiai</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Kamil</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Walukiewicz</t>
+          <t>Wiktorski</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>[Włochy] US Sassuolo</t>
+          <t>[Rumunia] CSC 1599 Selimbar</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Jakub</t>
+          <t>Szymon</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Wawszczyk</t>
+          <t>Wlodarczyk</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>[Litwa] FC Džiugas Telšiai</t>
+          <t>[Austria] SK Sturm Graz</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Kamil</t>
+          <t>Oskar</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Wiktorski</t>
+          <t>Wójcik</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>[Rumunia] CSC 1599 Selimbar</t>
+          <t>[Niemcy] SV Werder Bremen</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Szymon</t>
+          <t>Nicola</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Wlodarczyk</t>
+          <t>Zalewski</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>[Austria] SK Sturm Graz</t>
+          <t>[Włochy] Atalanta BC</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Oskar</t>
+          <t>Marcel</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Wójcik</t>
+          <t>Zapytowski</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>[Niemcy] SV Werder Bremen</t>
+          <t>[Norwegia] Egersunds IK</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Nicola</t>
+          <t>Oskar</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Zalewski</t>
+          <t>Zawada</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>[Włochy] Atalanta BC</t>
+          <t>[Holandia] FC Groningen</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Marcel</t>
+          <t>Alan</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Zapytowski</t>
+          <t>Zborowski</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>[Norwegia] Egersunds IK</t>
+          <t>[Irlandia] Cobh Ramblers FC</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Oskar</t>
+          <t>Jakub</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Zawada</t>
+          <t>Zieliński</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>[Holandia] FC Groningen</t>
+          <t>[Niemcy] VfL Wolfsburg</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Alan</t>
+          <t>Piotr</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Zborowski</t>
+          <t>Zieliński</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>[Irlandia] Cobh Ramblers FC</t>
+          <t>[Włochy] Inter Mediolan</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Piotr</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Zielinski</t>
+          <t>Ziolkowski</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>[Włochy] Inter Mediolan</t>
+          <t>[Włochy] AC Monza</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Jakub</t>
+          <t>Mateusz</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Zieliński</t>
+          <t>Zukowski</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>[Niemcy] VfL Wolfsburg</t>
+          <t>[Niemcy] 1.FC Magdeburg</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Łukasz</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Ziolkowski</t>
+          <t>Zwoliński</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>[Włochy] AC Monza</t>
+          <t>[Indie] East Bengal FC</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Mateusz</t>
+          <t>Oliwier</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Zukowski</t>
+          <t>Zych</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
-        <is>
-          <t>[Niemcy] 1.FC Magdeburg</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>Łukasz</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>Zwoliński</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>[Indie] East Bengal FC</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>Oliwier</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>Zych</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
         <is>
           <t>[Portugalia] Vitoria Guimarães SC</t>
         </is>

</xml_diff>